<commit_message>
inclusao de fotos carrossel, links mercado pago
</commit_message>
<xml_diff>
--- a/convidados Atualizado.xlsx
+++ b/convidados Atualizado.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kenji\Documents\casamento-react-firebase\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02129F13-431C-42A4-8971-79F738BDC7A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{502C7D8E-1565-4986-9A38-801858447577}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="16663" windowHeight="8743" xr2:uid="{2618C885-8054-4ACF-AD14-453306E82E46}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$F$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$K$104</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="221">
   <si>
     <t>Nome</t>
   </si>
@@ -720,7 +720,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -739,6 +739,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -752,152 +758,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="17">
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1227,6 +1097,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95DA610D-7716-4AEA-B8A6-BF53A20C5BB8}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:K104"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
@@ -1273,7 +1144,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>190</v>
       </c>
@@ -1284,7 +1155,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>190</v>
       </c>
@@ -1295,7 +1166,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>190</v>
       </c>
@@ -1303,7 +1174,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>190</v>
       </c>
@@ -1311,7 +1182,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>190</v>
       </c>
@@ -1322,7 +1193,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:11" hidden="1" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>190</v>
       </c>
@@ -1330,7 +1201,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>190</v>
       </c>
@@ -1338,7 +1209,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>190</v>
       </c>
@@ -1346,7 +1217,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:11" hidden="1" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>190</v>
       </c>
@@ -1357,7 +1228,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:11" hidden="1" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>190</v>
       </c>
@@ -1368,7 +1239,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:11" hidden="1" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>190</v>
       </c>
@@ -1379,7 +1250,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:11" hidden="1" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>190</v>
       </c>
@@ -1390,7 +1261,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:11" hidden="1" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>190</v>
       </c>
@@ -1401,7 +1272,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>190</v>
       </c>
@@ -1412,7 +1283,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:11" hidden="1" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>190</v>
       </c>
@@ -1420,7 +1291,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>190</v>
       </c>
@@ -1428,7 +1299,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>190</v>
       </c>
@@ -1439,7 +1310,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>190</v>
       </c>
@@ -1456,7 +1327,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>190</v>
       </c>
@@ -1464,7 +1335,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>190</v>
       </c>
@@ -1472,7 +1343,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>190</v>
       </c>
@@ -1503,55 +1374,55 @@
         <v>160</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A24" t="s">
+    <row r="24" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A25" t="s">
+    <row r="25" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A26" t="s">
+    <row r="26" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A27" t="s">
+    <row r="27" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A27" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A28" t="s">
+    <row r="28" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A28" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="3" t="s">
         <v>113</v>
       </c>
     </row>
@@ -1649,7 +1520,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>33</v>
       </c>
@@ -1660,7 +1531,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
         <v>33</v>
       </c>
@@ -1674,7 +1545,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
         <v>33</v>
       </c>
@@ -1685,7 +1556,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
         <v>33</v>
       </c>
@@ -1696,7 +1567,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
         <v>33</v>
       </c>
@@ -1707,7 +1578,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>33</v>
       </c>
@@ -1721,7 +1592,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A43" t="s">
         <v>33</v>
       </c>
@@ -1732,7 +1603,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
         <v>33</v>
       </c>
@@ -1743,7 +1614,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
         <v>33</v>
       </c>
@@ -1754,7 +1625,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A46" t="s">
         <v>33</v>
       </c>
@@ -1771,7 +1642,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A47" t="s">
         <v>33</v>
       </c>
@@ -1785,7 +1656,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A48" t="s">
         <v>33</v>
       </c>
@@ -1799,7 +1670,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A49" t="s">
         <v>33</v>
       </c>
@@ -1810,7 +1681,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A50" t="s">
         <v>33</v>
       </c>
@@ -1821,7 +1692,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
         <v>33</v>
       </c>
@@ -1841,7 +1712,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
         <v>33</v>
       </c>
@@ -1849,7 +1720,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
         <v>33</v>
       </c>
@@ -1857,7 +1728,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
         <v>33</v>
       </c>
@@ -1871,7 +1742,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
         <v>33</v>
       </c>
@@ -1885,7 +1756,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A56" t="s">
         <v>33</v>
       </c>
@@ -1902,7 +1773,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A57" t="s">
         <v>33</v>
       </c>
@@ -1913,7 +1784,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A58" t="s">
         <v>33</v>
       </c>
@@ -1927,7 +1798,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A59" t="s">
         <v>33</v>
       </c>
@@ -1935,7 +1806,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A60" t="s">
         <v>33</v>
       </c>
@@ -1943,7 +1814,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A61" t="s">
         <v>33</v>
       </c>
@@ -1954,7 +1825,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A62" t="s">
         <v>33</v>
       </c>
@@ -1965,7 +1836,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A63" t="s">
         <v>33</v>
       </c>
@@ -1976,7 +1847,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A64" t="s">
         <v>33</v>
       </c>
@@ -1993,7 +1864,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A65" t="s">
         <v>33</v>
       </c>
@@ -2001,7 +1872,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A66" t="s">
         <v>33</v>
       </c>
@@ -2009,7 +1880,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A67" t="s">
         <v>191</v>
       </c>
@@ -2020,7 +1891,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A68" t="s">
         <v>191</v>
       </c>
@@ -2031,7 +1902,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A69" t="s">
         <v>191</v>
       </c>
@@ -2042,7 +1913,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A70" t="s">
         <v>191</v>
       </c>
@@ -2053,7 +1924,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A71" t="s">
         <v>191</v>
       </c>
@@ -2067,7 +1938,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A72" t="s">
         <v>191</v>
       </c>
@@ -2078,7 +1949,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A73" t="s">
         <v>191</v>
       </c>
@@ -2089,7 +1960,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A74" t="s">
         <v>191</v>
       </c>
@@ -2100,7 +1971,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A75" t="s">
         <v>191</v>
       </c>
@@ -2111,7 +1982,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A76" t="s">
         <v>191</v>
       </c>
@@ -2122,7 +1993,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A77" t="s">
         <v>191</v>
       </c>
@@ -2133,7 +2004,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A78" t="s">
         <v>191</v>
       </c>
@@ -2141,7 +2012,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A79" t="s">
         <v>189</v>
       </c>
@@ -2152,7 +2023,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="A80" t="s">
         <v>189</v>
       </c>
@@ -2169,7 +2040,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:4" hidden="1" x14ac:dyDescent="0.4">
       <c r="A81" t="s">
         <v>189</v>
       </c>
@@ -2180,7 +2051,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:4" hidden="1" x14ac:dyDescent="0.4">
       <c r="A82" t="s">
         <v>189</v>
       </c>
@@ -2191,7 +2062,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:4" hidden="1" x14ac:dyDescent="0.4">
       <c r="A83" t="s">
         <v>189</v>
       </c>
@@ -2205,7 +2076,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="84" spans="1:4" hidden="1" x14ac:dyDescent="0.4">
       <c r="A84" t="s">
         <v>189</v>
       </c>
@@ -2216,7 +2087,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:4" hidden="1" x14ac:dyDescent="0.4">
       <c r="A85" t="s">
         <v>189</v>
       </c>
@@ -2227,7 +2098,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:4" hidden="1" x14ac:dyDescent="0.4">
       <c r="A86" t="s">
         <v>189</v>
       </c>
@@ -2238,7 +2109,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:4" hidden="1" x14ac:dyDescent="0.4">
       <c r="A87" t="s">
         <v>189</v>
       </c>
@@ -2246,7 +2117,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="88" spans="1:4" hidden="1" x14ac:dyDescent="0.4">
       <c r="A88" t="s">
         <v>189</v>
       </c>
@@ -2254,7 +2125,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:4" hidden="1" x14ac:dyDescent="0.4">
       <c r="A89" t="s">
         <v>189</v>
       </c>
@@ -2265,7 +2136,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="90" spans="1:4" hidden="1" x14ac:dyDescent="0.4">
       <c r="A90" t="s">
         <v>192</v>
       </c>
@@ -2276,7 +2147,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="91" spans="1:4" hidden="1" x14ac:dyDescent="0.4">
       <c r="A91" t="s">
         <v>192</v>
       </c>
@@ -2287,7 +2158,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="92" spans="1:4" hidden="1" x14ac:dyDescent="0.4">
       <c r="A92" t="s">
         <v>192</v>
       </c>
@@ -2298,7 +2169,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:4" hidden="1" x14ac:dyDescent="0.4">
       <c r="A93" t="s">
         <v>192</v>
       </c>
@@ -2307,7 +2178,7 @@
       </c>
       <c r="C93" s="1"/>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="94" spans="1:4" hidden="1" x14ac:dyDescent="0.4">
       <c r="A94" t="s">
         <v>192</v>
       </c>
@@ -2316,7 +2187,7 @@
       </c>
       <c r="C94" s="1"/>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="95" spans="1:4" hidden="1" x14ac:dyDescent="0.4">
       <c r="A95" t="s">
         <v>192</v>
       </c>
@@ -2327,7 +2198,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="96" spans="1:4" hidden="1" x14ac:dyDescent="0.4">
       <c r="A96" t="s">
         <v>192</v>
       </c>
@@ -2338,7 +2209,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="97" spans="1:3" hidden="1" x14ac:dyDescent="0.4">
       <c r="A97" t="s">
         <v>192</v>
       </c>
@@ -2349,7 +2220,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="98" spans="1:3" hidden="1" x14ac:dyDescent="0.4">
       <c r="A98" t="s">
         <v>33</v>
       </c>
@@ -2380,7 +2251,7 @@
       </c>
       <c r="C100" s="1"/>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="101" spans="1:3" hidden="1" x14ac:dyDescent="0.4">
       <c r="A101" t="s">
         <v>189</v>
       </c>
@@ -2419,6 +2290,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:K104" xr:uid="{95DA610D-7716-4AEA-B8A6-BF53A20C5BB8}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Grupo Noiva"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>